<commit_message>
LATEST UPDATE, ADDED OTHER TEACHERS AND MODIFIED TEMPLATES
</commit_message>
<xml_diff>
--- a/resources/templates/SAMPLE MONITORING.xlsx
+++ b/resources/templates/SAMPLE MONITORING.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="8400"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="SAMPLE" sheetId="14" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SAMPLE!$A$2:$AO$450</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">SAMPLE!$A$2:$AO$452</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="70">
   <si>
     <t>ODC NO.</t>
   </si>
@@ -170,7 +170,7 @@
     <t>${position}</t>
   </si>
   <si>
-    <t>${vice}</t>
+    <t>${employee_name}</t>
   </si>
   <si>
     <t>${sex}</t>
@@ -219,6 +219,9 @@
   </si>
   <si>
     <t>${ethnicity}</t>
+  </si>
+  <si>
+    <t>${vice}</t>
   </si>
   <si>
     <t>${natural_vacancy}</t>
@@ -1724,7 +1727,7 @@
     <tabColor theme="9" tint="0.599993896298105"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AP518"/>
+  <dimension ref="A1:AP520"/>
   <sheetFormatPr defaultColWidth="12.5740740740741" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="20" style="1" customWidth="1"/>
@@ -1998,10 +2001,10 @@
         <v>62</v>
       </c>
       <c r="Y3" s="35" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="Z3" s="35" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="AA3" s="38"/>
       <c r="AB3" s="38"/>
@@ -2015,10 +2018,10 @@
       <c r="AJ3" s="34"/>
       <c r="AK3" s="34"/>
       <c r="AL3" s="34" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM3" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="AN3" s="40"/>
       <c r="AO3" s="40"/>
@@ -2063,10 +2066,10 @@
       <c r="AJ4" s="50"/>
       <c r="AK4" s="50"/>
       <c r="AL4" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM4" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" s="2" customFormat="1" customHeight="1" spans="1:42">
@@ -2108,10 +2111,10 @@
       <c r="AJ5" s="50"/>
       <c r="AK5" s="50"/>
       <c r="AL5" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM5" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" s="2" customFormat="1" customHeight="1" spans="1:42">
@@ -2153,10 +2156,10 @@
       <c r="AJ6" s="50"/>
       <c r="AK6" s="50"/>
       <c r="AL6" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM6" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" s="2" customFormat="1" customHeight="1" spans="1:42">
@@ -2198,10 +2201,10 @@
       <c r="AJ7" s="50"/>
       <c r="AK7" s="50"/>
       <c r="AL7" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM7" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" s="2" customFormat="1" customHeight="1" spans="1:42">
@@ -2243,10 +2246,10 @@
       <c r="AJ8" s="50"/>
       <c r="AK8" s="50"/>
       <c r="AL8" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM8" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" s="2" customFormat="1" customHeight="1" spans="1:42">
@@ -2288,10 +2291,10 @@
       <c r="AJ9" s="50"/>
       <c r="AK9" s="50"/>
       <c r="AL9" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM9" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" s="2" customFormat="1" customHeight="1" spans="1:42">
@@ -2333,10 +2336,10 @@
       <c r="AJ10" s="50"/>
       <c r="AK10" s="50"/>
       <c r="AL10" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM10" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" s="2" customFormat="1" customHeight="1" spans="1:42">
@@ -2378,10 +2381,10 @@
       <c r="AJ11" s="50"/>
       <c r="AK11" s="50"/>
       <c r="AL11" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM11" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" s="2" customFormat="1" customHeight="1" spans="1:42">
@@ -2423,10 +2426,10 @@
       <c r="AJ12" s="50"/>
       <c r="AK12" s="50"/>
       <c r="AL12" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM12" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" s="2" customFormat="1" customHeight="1" spans="1:42">
@@ -2468,10 +2471,10 @@
       <c r="AJ13" s="50"/>
       <c r="AK13" s="50"/>
       <c r="AL13" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM13" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" s="2" customFormat="1" customHeight="1" spans="1:42">
@@ -2513,10 +2516,10 @@
       <c r="AJ14" s="50"/>
       <c r="AK14" s="50"/>
       <c r="AL14" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM14" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" s="2" customFormat="1" customHeight="1" spans="1:42">
@@ -2558,10 +2561,10 @@
       <c r="AJ15" s="50"/>
       <c r="AK15" s="50"/>
       <c r="AL15" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM15" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" s="2" customFormat="1" customHeight="1" spans="1:42">
@@ -2603,10 +2606,10 @@
       <c r="AJ16" s="50"/>
       <c r="AK16" s="50"/>
       <c r="AL16" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM16" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -2648,10 +2651,10 @@
       <c r="AJ17" s="50"/>
       <c r="AK17" s="50"/>
       <c r="AL17" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM17" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -2693,10 +2696,10 @@
       <c r="AJ18" s="50"/>
       <c r="AK18" s="50"/>
       <c r="AL18" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM18" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -2737,12 +2740,8 @@
       <c r="AI19" s="50"/>
       <c r="AJ19" s="50"/>
       <c r="AK19" s="50"/>
-      <c r="AL19" s="39" t="s">
-        <v>64</v>
-      </c>
-      <c r="AM19" s="39" t="s">
-        <v>65</v>
-      </c>
+      <c r="AL19" s="39"/>
+      <c r="AM19" s="39"/>
     </row>
     <row r="20" s="2" customFormat="1" customHeight="1" spans="1:39">
       <c r="A20" s="41"/>
@@ -2782,60 +2781,52 @@
       <c r="AI20" s="50"/>
       <c r="AJ20" s="50"/>
       <c r="AK20" s="50"/>
-      <c r="AL20" s="39" t="s">
-        <v>64</v>
-      </c>
-      <c r="AM20" s="39" t="s">
+      <c r="AL20" s="39"/>
+      <c r="AM20" s="39"/>
+    </row>
+    <row r="21" s="2" customFormat="1" customHeight="1" spans="1:39">
+      <c r="A21" s="41"/>
+      <c r="B21" s="45"/>
+      <c r="C21" s="45"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="43"/>
+      <c r="I21" s="44"/>
+      <c r="J21" s="45"/>
+      <c r="K21" s="41"/>
+      <c r="L21" s="45"/>
+      <c r="M21" s="45"/>
+      <c r="N21" s="46"/>
+      <c r="O21" s="45"/>
+      <c r="P21" s="47"/>
+      <c r="Q21" s="32"/>
+      <c r="R21" s="47"/>
+      <c r="S21" s="47"/>
+      <c r="T21" s="47"/>
+      <c r="U21" s="32"/>
+      <c r="V21" s="48"/>
+      <c r="W21" s="48"/>
+      <c r="X21" s="48"/>
+      <c r="Y21" s="41"/>
+      <c r="Z21" s="41"/>
+      <c r="AA21" s="49"/>
+      <c r="AB21" s="49"/>
+      <c r="AC21" s="49"/>
+      <c r="AD21" s="49"/>
+      <c r="AE21" s="45"/>
+      <c r="AF21" s="45"/>
+      <c r="AG21" s="50"/>
+      <c r="AH21" s="50"/>
+      <c r="AI21" s="50"/>
+      <c r="AJ21" s="50"/>
+      <c r="AK21" s="50"/>
+      <c r="AL21" s="39" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="21" s="3" customFormat="1" customHeight="1" spans="1:39">
-      <c r="A21" s="52"/>
-      <c r="B21" s="53"/>
-      <c r="C21" s="53"/>
-      <c r="D21" s="52"/>
-      <c r="E21" s="54"/>
-      <c r="F21" s="52"/>
-      <c r="G21" s="52"/>
-      <c r="H21" s="55"/>
-      <c r="I21" s="56"/>
-      <c r="J21" s="53"/>
-      <c r="K21" s="52"/>
-      <c r="L21" s="53"/>
-      <c r="M21" s="53"/>
-      <c r="N21" s="57"/>
-      <c r="O21" s="53"/>
-      <c r="P21" s="58"/>
-      <c r="Q21" s="59"/>
-      <c r="R21" s="58"/>
-      <c r="S21" s="58"/>
-      <c r="T21" s="58"/>
-      <c r="U21" s="59"/>
-      <c r="V21" s="60"/>
-      <c r="W21" s="60"/>
-      <c r="X21" s="60"/>
-      <c r="Y21" s="52"/>
-      <c r="Z21" s="52"/>
-      <c r="AA21" s="61"/>
-      <c r="AB21" s="61"/>
-      <c r="AC21" s="61"/>
-      <c r="AD21" s="61"/>
-      <c r="AE21" s="109" t="s">
+      <c r="AM21" s="39" t="s">
         <v>66</v>
-      </c>
-      <c r="AF21" s="109" t="s">
-        <v>67</v>
-      </c>
-      <c r="AG21" s="62"/>
-      <c r="AH21" s="62"/>
-      <c r="AI21" s="62"/>
-      <c r="AJ21" s="62"/>
-      <c r="AK21" s="62"/>
-      <c r="AL21" s="39" t="s">
-        <v>64</v>
-      </c>
-      <c r="AM21" s="39" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="22" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -2877,58 +2868,62 @@
       <c r="AJ22" s="50"/>
       <c r="AK22" s="50"/>
       <c r="AL22" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM22" s="39" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" s="3" customFormat="1" customHeight="1" spans="1:39">
+      <c r="A23" s="52"/>
+      <c r="B23" s="53"/>
+      <c r="C23" s="53"/>
+      <c r="D23" s="52"/>
+      <c r="E23" s="54"/>
+      <c r="F23" s="52"/>
+      <c r="G23" s="52"/>
+      <c r="H23" s="55"/>
+      <c r="I23" s="56"/>
+      <c r="J23" s="53"/>
+      <c r="K23" s="52"/>
+      <c r="L23" s="53"/>
+      <c r="M23" s="53"/>
+      <c r="N23" s="57"/>
+      <c r="O23" s="53"/>
+      <c r="P23" s="58"/>
+      <c r="Q23" s="59"/>
+      <c r="R23" s="58"/>
+      <c r="S23" s="58"/>
+      <c r="T23" s="58"/>
+      <c r="U23" s="59"/>
+      <c r="V23" s="60"/>
+      <c r="W23" s="60"/>
+      <c r="X23" s="60"/>
+      <c r="Y23" s="52"/>
+      <c r="Z23" s="52"/>
+      <c r="AA23" s="61"/>
+      <c r="AB23" s="61"/>
+      <c r="AC23" s="61"/>
+      <c r="AD23" s="61"/>
+      <c r="AE23" s="109" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF23" s="109" t="s">
+        <v>68</v>
+      </c>
+      <c r="AG23" s="62"/>
+      <c r="AH23" s="62"/>
+      <c r="AI23" s="62"/>
+      <c r="AJ23" s="62"/>
+      <c r="AK23" s="62"/>
+      <c r="AL23" s="39" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="23" s="2" customFormat="1" customHeight="1" spans="1:39">
-      <c r="A23" s="41"/>
-      <c r="B23" s="45"/>
-      <c r="C23" s="45"/>
-      <c r="D23" s="41"/>
-      <c r="E23" s="42"/>
-      <c r="F23" s="41"/>
-      <c r="G23" s="41"/>
-      <c r="H23" s="43"/>
-      <c r="I23" s="44"/>
-      <c r="J23" s="45"/>
-      <c r="K23" s="41"/>
-      <c r="L23" s="45"/>
-      <c r="M23" s="45"/>
-      <c r="N23" s="46"/>
-      <c r="O23" s="45"/>
-      <c r="P23" s="47"/>
-      <c r="Q23" s="32"/>
-      <c r="R23" s="47"/>
-      <c r="S23" s="47"/>
-      <c r="T23" s="47"/>
-      <c r="U23" s="32"/>
-      <c r="V23" s="48"/>
-      <c r="W23" s="48"/>
-      <c r="X23" s="48"/>
-      <c r="Y23" s="41"/>
-      <c r="Z23" s="41"/>
-      <c r="AA23" s="49"/>
-      <c r="AB23" s="49"/>
-      <c r="AC23" s="49"/>
-      <c r="AD23" s="49"/>
-      <c r="AE23" s="45"/>
-      <c r="AF23" s="45"/>
-      <c r="AG23" s="50"/>
-      <c r="AH23" s="50"/>
-      <c r="AI23" s="50"/>
-      <c r="AJ23" s="50"/>
-      <c r="AK23" s="50"/>
-      <c r="AL23" s="39" t="s">
-        <v>64</v>
-      </c>
       <c r="AM23" s="39" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="24" s="2" customFormat="1" ht="14.25" customHeight="1" spans="1:39">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="24" s="2" customFormat="1" customHeight="1" spans="1:39">
       <c r="A24" s="41"/>
       <c r="B24" s="45"/>
       <c r="C24" s="45"/>
@@ -2967,10 +2962,10 @@
       <c r="AJ24" s="50"/>
       <c r="AK24" s="50"/>
       <c r="AL24" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM24" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -3012,13 +3007,13 @@
       <c r="AJ25" s="50"/>
       <c r="AK25" s="50"/>
       <c r="AL25" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM25" s="39" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="26" s="2" customFormat="1" customHeight="1" spans="1:39">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" s="2" customFormat="1" ht="14.25" customHeight="1" spans="1:39">
       <c r="A26" s="41"/>
       <c r="B26" s="45"/>
       <c r="C26" s="45"/>
@@ -3057,10 +3052,10 @@
       <c r="AJ26" s="50"/>
       <c r="AK26" s="50"/>
       <c r="AL26" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM26" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -3080,7 +3075,7 @@
       <c r="N27" s="46"/>
       <c r="O27" s="45"/>
       <c r="P27" s="47"/>
-      <c r="Q27" s="51"/>
+      <c r="Q27" s="32"/>
       <c r="R27" s="47"/>
       <c r="S27" s="47"/>
       <c r="T27" s="47"/>
@@ -3102,10 +3097,10 @@
       <c r="AJ27" s="50"/>
       <c r="AK27" s="50"/>
       <c r="AL27" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM27" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -3125,7 +3120,7 @@
       <c r="N28" s="46"/>
       <c r="O28" s="45"/>
       <c r="P28" s="47"/>
-      <c r="Q28" s="51"/>
+      <c r="Q28" s="32"/>
       <c r="R28" s="47"/>
       <c r="S28" s="47"/>
       <c r="T28" s="47"/>
@@ -3147,10 +3142,10 @@
       <c r="AJ28" s="50"/>
       <c r="AK28" s="50"/>
       <c r="AL28" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM28" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -3192,10 +3187,10 @@
       <c r="AJ29" s="50"/>
       <c r="AK29" s="50"/>
       <c r="AL29" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM29" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="30" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -3237,10 +3232,10 @@
       <c r="AJ30" s="50"/>
       <c r="AK30" s="50"/>
       <c r="AL30" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM30" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="31" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -3282,20 +3277,20 @@
       <c r="AJ31" s="50"/>
       <c r="AK31" s="50"/>
       <c r="AL31" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM31" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="32" s="2" customFormat="1" customHeight="1" spans="1:39">
-      <c r="A32" s="32"/>
+      <c r="A32" s="41"/>
       <c r="B32" s="45"/>
       <c r="C32" s="45"/>
       <c r="D32" s="41"/>
       <c r="E32" s="42"/>
-      <c r="F32" s="32"/>
-      <c r="G32" s="32"/>
+      <c r="F32" s="41"/>
+      <c r="G32" s="41"/>
       <c r="H32" s="43"/>
       <c r="I32" s="44"/>
       <c r="J32" s="45"/>
@@ -3305,8 +3300,8 @@
       <c r="N32" s="46"/>
       <c r="O32" s="45"/>
       <c r="P32" s="47"/>
-      <c r="Q32" s="63"/>
-      <c r="R32" s="63"/>
+      <c r="Q32" s="51"/>
+      <c r="R32" s="47"/>
       <c r="S32" s="47"/>
       <c r="T32" s="47"/>
       <c r="U32" s="32"/>
@@ -3327,14 +3322,14 @@
       <c r="AJ32" s="50"/>
       <c r="AK32" s="50"/>
       <c r="AL32" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM32" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="33" s="2" customFormat="1" customHeight="1" spans="1:39">
-      <c r="A33" s="32"/>
+      <c r="A33" s="41"/>
       <c r="B33" s="45"/>
       <c r="C33" s="45"/>
       <c r="D33" s="41"/>
@@ -3350,8 +3345,8 @@
       <c r="N33" s="46"/>
       <c r="O33" s="45"/>
       <c r="P33" s="47"/>
-      <c r="Q33" s="63"/>
-      <c r="R33" s="63"/>
+      <c r="Q33" s="51"/>
+      <c r="R33" s="47"/>
       <c r="S33" s="47"/>
       <c r="T33" s="47"/>
       <c r="U33" s="32"/>
@@ -3372,20 +3367,20 @@
       <c r="AJ33" s="50"/>
       <c r="AK33" s="50"/>
       <c r="AL33" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM33" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="34" s="2" customFormat="1" customHeight="1" spans="1:39">
-      <c r="A34" s="41"/>
+      <c r="A34" s="32"/>
       <c r="B34" s="45"/>
       <c r="C34" s="45"/>
       <c r="D34" s="41"/>
       <c r="E34" s="42"/>
-      <c r="F34" s="41"/>
-      <c r="G34" s="41"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="32"/>
       <c r="H34" s="43"/>
       <c r="I34" s="44"/>
       <c r="J34" s="45"/>
@@ -3395,7 +3390,7 @@
       <c r="N34" s="46"/>
       <c r="O34" s="45"/>
       <c r="P34" s="47"/>
-      <c r="Q34" s="51"/>
+      <c r="Q34" s="63"/>
       <c r="R34" s="63"/>
       <c r="S34" s="47"/>
       <c r="T34" s="47"/>
@@ -3417,14 +3412,14 @@
       <c r="AJ34" s="50"/>
       <c r="AK34" s="50"/>
       <c r="AL34" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM34" s="39" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="35" s="2" customFormat="1" ht="14.25" customHeight="1" spans="1:39">
-      <c r="A35" s="41"/>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="35" s="2" customFormat="1" customHeight="1" spans="1:39">
+      <c r="A35" s="32"/>
       <c r="B35" s="45"/>
       <c r="C35" s="45"/>
       <c r="D35" s="41"/>
@@ -3440,7 +3435,7 @@
       <c r="N35" s="46"/>
       <c r="O35" s="45"/>
       <c r="P35" s="47"/>
-      <c r="Q35" s="51"/>
+      <c r="Q35" s="63"/>
       <c r="R35" s="63"/>
       <c r="S35" s="47"/>
       <c r="T35" s="47"/>
@@ -3462,10 +3457,10 @@
       <c r="AJ35" s="50"/>
       <c r="AK35" s="50"/>
       <c r="AL35" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM35" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="36" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -3507,13 +3502,13 @@
       <c r="AJ36" s="50"/>
       <c r="AK36" s="50"/>
       <c r="AL36" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM36" s="39" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="37" s="2" customFormat="1" customHeight="1" spans="1:39">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="37" s="2" customFormat="1" ht="14.25" customHeight="1" spans="1:39">
       <c r="A37" s="41"/>
       <c r="B37" s="45"/>
       <c r="C37" s="45"/>
@@ -3530,7 +3525,7 @@
       <c r="N37" s="46"/>
       <c r="O37" s="45"/>
       <c r="P37" s="47"/>
-      <c r="Q37" s="63"/>
+      <c r="Q37" s="51"/>
       <c r="R37" s="63"/>
       <c r="S37" s="47"/>
       <c r="T37" s="47"/>
@@ -3552,10 +3547,10 @@
       <c r="AJ37" s="50"/>
       <c r="AK37" s="50"/>
       <c r="AL37" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM37" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="38" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -3597,10 +3592,10 @@
       <c r="AJ38" s="50"/>
       <c r="AK38" s="50"/>
       <c r="AL38" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM38" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="39" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -3620,7 +3615,7 @@
       <c r="N39" s="46"/>
       <c r="O39" s="45"/>
       <c r="P39" s="47"/>
-      <c r="Q39" s="51"/>
+      <c r="Q39" s="63"/>
       <c r="R39" s="63"/>
       <c r="S39" s="47"/>
       <c r="T39" s="47"/>
@@ -3642,10 +3637,10 @@
       <c r="AJ39" s="50"/>
       <c r="AK39" s="50"/>
       <c r="AL39" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM39" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="40" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -3687,100 +3682,100 @@
       <c r="AJ40" s="50"/>
       <c r="AK40" s="50"/>
       <c r="AL40" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM40" s="39" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="41" customHeight="1" spans="1:39">
-      <c r="A41" s="64"/>
-      <c r="B41" s="65"/>
-      <c r="C41" s="65"/>
-      <c r="D41" s="64"/>
-      <c r="E41" s="66"/>
-      <c r="F41" s="64"/>
-      <c r="G41" s="64"/>
-      <c r="H41" s="67"/>
-      <c r="I41" s="68"/>
-      <c r="J41" s="65"/>
-      <c r="K41" s="64"/>
-      <c r="L41" s="65"/>
-      <c r="M41" s="65"/>
-      <c r="N41" s="69"/>
-      <c r="O41" s="65"/>
-      <c r="P41" s="70"/>
-      <c r="Q41" s="71"/>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="41" s="2" customFormat="1" customHeight="1" spans="1:39">
+      <c r="A41" s="41"/>
+      <c r="B41" s="45"/>
+      <c r="C41" s="45"/>
+      <c r="D41" s="41"/>
+      <c r="E41" s="42"/>
+      <c r="F41" s="41"/>
+      <c r="G41" s="41"/>
+      <c r="H41" s="43"/>
+      <c r="I41" s="44"/>
+      <c r="J41" s="45"/>
+      <c r="K41" s="41"/>
+      <c r="L41" s="45"/>
+      <c r="M41" s="45"/>
+      <c r="N41" s="46"/>
+      <c r="O41" s="45"/>
+      <c r="P41" s="47"/>
+      <c r="Q41" s="51"/>
       <c r="R41" s="63"/>
-      <c r="S41" s="70"/>
-      <c r="T41" s="70"/>
-      <c r="U41" s="72"/>
+      <c r="S41" s="47"/>
+      <c r="T41" s="47"/>
+      <c r="U41" s="32"/>
       <c r="V41" s="48"/>
       <c r="W41" s="48"/>
       <c r="X41" s="48"/>
-      <c r="Y41" s="64"/>
-      <c r="Z41" s="64"/>
-      <c r="AA41" s="73"/>
-      <c r="AB41" s="73"/>
-      <c r="AC41" s="73"/>
-      <c r="AD41" s="73"/>
-      <c r="AE41" s="65"/>
-      <c r="AF41" s="65"/>
-      <c r="AG41" s="74"/>
-      <c r="AH41" s="74"/>
-      <c r="AI41" s="74"/>
-      <c r="AJ41" s="74"/>
-      <c r="AK41" s="74"/>
+      <c r="Y41" s="41"/>
+      <c r="Z41" s="41"/>
+      <c r="AA41" s="49"/>
+      <c r="AB41" s="49"/>
+      <c r="AC41" s="49"/>
+      <c r="AD41" s="49"/>
+      <c r="AE41" s="45"/>
+      <c r="AF41" s="45"/>
+      <c r="AG41" s="50"/>
+      <c r="AH41" s="50"/>
+      <c r="AI41" s="50"/>
+      <c r="AJ41" s="50"/>
+      <c r="AK41" s="50"/>
       <c r="AL41" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM41" s="39" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="42" customHeight="1" spans="1:39">
-      <c r="A42" s="64"/>
-      <c r="B42" s="65"/>
-      <c r="C42" s="65"/>
-      <c r="D42" s="64"/>
-      <c r="E42" s="66"/>
-      <c r="F42" s="64"/>
-      <c r="G42" s="64"/>
-      <c r="H42" s="67"/>
-      <c r="I42" s="68"/>
-      <c r="J42" s="65"/>
-      <c r="K42" s="64"/>
-      <c r="L42" s="65"/>
-      <c r="M42" s="65"/>
-      <c r="N42" s="69"/>
-      <c r="O42" s="65"/>
-      <c r="P42" s="70"/>
-      <c r="Q42" s="71"/>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="42" s="2" customFormat="1" customHeight="1" spans="1:39">
+      <c r="A42" s="41"/>
+      <c r="B42" s="45"/>
+      <c r="C42" s="45"/>
+      <c r="D42" s="41"/>
+      <c r="E42" s="42"/>
+      <c r="F42" s="41"/>
+      <c r="G42" s="41"/>
+      <c r="H42" s="43"/>
+      <c r="I42" s="44"/>
+      <c r="J42" s="45"/>
+      <c r="K42" s="41"/>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
+      <c r="N42" s="46"/>
+      <c r="O42" s="45"/>
+      <c r="P42" s="47"/>
+      <c r="Q42" s="51"/>
       <c r="R42" s="63"/>
-      <c r="S42" s="70"/>
-      <c r="T42" s="70"/>
-      <c r="U42" s="72"/>
+      <c r="S42" s="47"/>
+      <c r="T42" s="47"/>
+      <c r="U42" s="32"/>
       <c r="V42" s="48"/>
       <c r="W42" s="48"/>
       <c r="X42" s="48"/>
-      <c r="Y42" s="64"/>
-      <c r="Z42" s="64"/>
-      <c r="AA42" s="73"/>
-      <c r="AB42" s="73"/>
-      <c r="AC42" s="73"/>
-      <c r="AD42" s="73"/>
-      <c r="AE42" s="65"/>
-      <c r="AF42" s="65"/>
-      <c r="AG42" s="74"/>
-      <c r="AH42" s="74"/>
-      <c r="AI42" s="74"/>
-      <c r="AJ42" s="74"/>
-      <c r="AK42" s="74"/>
+      <c r="Y42" s="41"/>
+      <c r="Z42" s="41"/>
+      <c r="AA42" s="49"/>
+      <c r="AB42" s="49"/>
+      <c r="AC42" s="49"/>
+      <c r="AD42" s="49"/>
+      <c r="AE42" s="45"/>
+      <c r="AF42" s="45"/>
+      <c r="AG42" s="50"/>
+      <c r="AH42" s="50"/>
+      <c r="AI42" s="50"/>
+      <c r="AJ42" s="50"/>
+      <c r="AK42" s="50"/>
       <c r="AL42" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM42" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="43" customHeight="1" spans="1:39">
@@ -3800,7 +3795,7 @@
       <c r="N43" s="69"/>
       <c r="O43" s="65"/>
       <c r="P43" s="70"/>
-      <c r="Q43" s="63"/>
+      <c r="Q43" s="71"/>
       <c r="R43" s="63"/>
       <c r="S43" s="70"/>
       <c r="T43" s="70"/>
@@ -3822,10 +3817,10 @@
       <c r="AJ43" s="74"/>
       <c r="AK43" s="74"/>
       <c r="AL43" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM43" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="44" customHeight="1" spans="1:39">
@@ -3867,10 +3862,10 @@
       <c r="AJ44" s="74"/>
       <c r="AK44" s="74"/>
       <c r="AL44" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM44" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="45" customHeight="1" spans="1:39">
@@ -3912,10 +3907,10 @@
       <c r="AJ45" s="74"/>
       <c r="AK45" s="74"/>
       <c r="AL45" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM45" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="46" customHeight="1" spans="1:39">
@@ -3935,7 +3930,7 @@
       <c r="N46" s="69"/>
       <c r="O46" s="65"/>
       <c r="P46" s="70"/>
-      <c r="Q46" s="63"/>
+      <c r="Q46" s="71"/>
       <c r="R46" s="63"/>
       <c r="S46" s="70"/>
       <c r="T46" s="70"/>
@@ -3957,10 +3952,10 @@
       <c r="AJ46" s="74"/>
       <c r="AK46" s="74"/>
       <c r="AL46" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM46" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="47" customHeight="1" spans="1:39">
@@ -4002,10 +3997,10 @@
       <c r="AJ47" s="74"/>
       <c r="AK47" s="74"/>
       <c r="AL47" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM47" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="48" customHeight="1" spans="1:39">
@@ -4047,10 +4042,10 @@
       <c r="AJ48" s="74"/>
       <c r="AK48" s="74"/>
       <c r="AL48" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM48" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="49" customHeight="1" spans="1:39">
@@ -4070,7 +4065,7 @@
       <c r="N49" s="69"/>
       <c r="O49" s="65"/>
       <c r="P49" s="70"/>
-      <c r="Q49" s="71"/>
+      <c r="Q49" s="63"/>
       <c r="R49" s="63"/>
       <c r="S49" s="70"/>
       <c r="T49" s="70"/>
@@ -4092,10 +4087,10 @@
       <c r="AJ49" s="74"/>
       <c r="AK49" s="74"/>
       <c r="AL49" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM49" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="50" customHeight="1" spans="1:39">
@@ -4115,7 +4110,7 @@
       <c r="N50" s="69"/>
       <c r="O50" s="65"/>
       <c r="P50" s="70"/>
-      <c r="Q50" s="71"/>
+      <c r="Q50" s="63"/>
       <c r="R50" s="63"/>
       <c r="S50" s="70"/>
       <c r="T50" s="70"/>
@@ -4137,10 +4132,10 @@
       <c r="AJ50" s="74"/>
       <c r="AK50" s="74"/>
       <c r="AL50" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM50" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="51" customHeight="1" spans="1:39">
@@ -4182,10 +4177,10 @@
       <c r="AJ51" s="74"/>
       <c r="AK51" s="74"/>
       <c r="AL51" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM51" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="52" customHeight="1" spans="1:39">
@@ -4205,7 +4200,7 @@
       <c r="N52" s="69"/>
       <c r="O52" s="65"/>
       <c r="P52" s="70"/>
-      <c r="Q52" s="63"/>
+      <c r="Q52" s="71"/>
       <c r="R52" s="63"/>
       <c r="S52" s="70"/>
       <c r="T52" s="70"/>
@@ -4227,10 +4222,10 @@
       <c r="AJ52" s="74"/>
       <c r="AK52" s="74"/>
       <c r="AL52" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM52" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="53" customHeight="1" spans="1:39">
@@ -4250,7 +4245,7 @@
       <c r="N53" s="69"/>
       <c r="O53" s="65"/>
       <c r="P53" s="70"/>
-      <c r="Q53" s="63"/>
+      <c r="Q53" s="71"/>
       <c r="R53" s="63"/>
       <c r="S53" s="70"/>
       <c r="T53" s="70"/>
@@ -4272,10 +4267,10 @@
       <c r="AJ53" s="74"/>
       <c r="AK53" s="74"/>
       <c r="AL53" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM53" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="54" customHeight="1" spans="1:39">
@@ -4317,10 +4312,10 @@
       <c r="AJ54" s="74"/>
       <c r="AK54" s="74"/>
       <c r="AL54" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM54" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="55" customHeight="1" spans="1:39">
@@ -4362,10 +4357,10 @@
       <c r="AJ55" s="74"/>
       <c r="AK55" s="74"/>
       <c r="AL55" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM55" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="56" customHeight="1" spans="1:39">
@@ -4407,13 +4402,13 @@
       <c r="AJ56" s="74"/>
       <c r="AK56" s="74"/>
       <c r="AL56" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM56" s="39" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="57" ht="28.5" customHeight="1" spans="1:39">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="57" customHeight="1" spans="1:39">
       <c r="A57" s="64"/>
       <c r="B57" s="65"/>
       <c r="C57" s="65"/>
@@ -4439,7 +4434,7 @@
       <c r="W57" s="48"/>
       <c r="X57" s="48"/>
       <c r="Y57" s="64"/>
-      <c r="Z57" s="75"/>
+      <c r="Z57" s="64"/>
       <c r="AA57" s="73"/>
       <c r="AB57" s="73"/>
       <c r="AC57" s="73"/>
@@ -4452,100 +4447,100 @@
       <c r="AJ57" s="74"/>
       <c r="AK57" s="74"/>
       <c r="AL57" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM57" s="39" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="58" s="2" customFormat="1" customHeight="1" spans="1:39">
-      <c r="A58" s="41"/>
-      <c r="B58" s="45"/>
-      <c r="C58" s="45"/>
-      <c r="D58" s="41"/>
-      <c r="E58" s="42"/>
-      <c r="F58" s="41"/>
-      <c r="G58" s="41"/>
-      <c r="H58" s="43"/>
-      <c r="I58" s="44"/>
-      <c r="J58" s="45"/>
-      <c r="K58" s="41"/>
-      <c r="L58" s="45"/>
-      <c r="M58" s="45"/>
-      <c r="N58" s="46"/>
-      <c r="O58" s="45"/>
-      <c r="P58" s="47"/>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="58" customHeight="1" spans="1:39">
+      <c r="A58" s="64"/>
+      <c r="B58" s="65"/>
+      <c r="C58" s="65"/>
+      <c r="D58" s="64"/>
+      <c r="E58" s="66"/>
+      <c r="F58" s="64"/>
+      <c r="G58" s="64"/>
+      <c r="H58" s="67"/>
+      <c r="I58" s="68"/>
+      <c r="J58" s="65"/>
+      <c r="K58" s="64"/>
+      <c r="L58" s="65"/>
+      <c r="M58" s="65"/>
+      <c r="N58" s="69"/>
+      <c r="O58" s="65"/>
+      <c r="P58" s="70"/>
       <c r="Q58" s="63"/>
       <c r="R58" s="63"/>
-      <c r="S58" s="47"/>
-      <c r="T58" s="47"/>
-      <c r="U58" s="32"/>
+      <c r="S58" s="70"/>
+      <c r="T58" s="70"/>
+      <c r="U58" s="72"/>
       <c r="V58" s="48"/>
       <c r="W58" s="48"/>
       <c r="X58" s="48"/>
-      <c r="Y58" s="41"/>
-      <c r="Z58" s="41"/>
-      <c r="AA58" s="49"/>
-      <c r="AB58" s="49"/>
-      <c r="AC58" s="49"/>
-      <c r="AD58" s="49"/>
-      <c r="AE58" s="45"/>
-      <c r="AF58" s="45"/>
-      <c r="AG58" s="50"/>
-      <c r="AH58" s="50"/>
-      <c r="AI58" s="50"/>
-      <c r="AJ58" s="50"/>
-      <c r="AK58" s="50"/>
+      <c r="Y58" s="64"/>
+      <c r="Z58" s="64"/>
+      <c r="AA58" s="73"/>
+      <c r="AB58" s="73"/>
+      <c r="AC58" s="73"/>
+      <c r="AD58" s="73"/>
+      <c r="AE58" s="65"/>
+      <c r="AF58" s="65"/>
+      <c r="AG58" s="74"/>
+      <c r="AH58" s="74"/>
+      <c r="AI58" s="74"/>
+      <c r="AJ58" s="74"/>
+      <c r="AK58" s="74"/>
       <c r="AL58" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM58" s="39" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="59" s="2" customFormat="1" customHeight="1" spans="1:39">
-      <c r="A59" s="41"/>
-      <c r="B59" s="45"/>
-      <c r="C59" s="45"/>
-      <c r="D59" s="41"/>
-      <c r="E59" s="42"/>
-      <c r="F59" s="41"/>
-      <c r="G59" s="41"/>
-      <c r="H59" s="43"/>
-      <c r="I59" s="44"/>
-      <c r="J59" s="45"/>
-      <c r="K59" s="41"/>
-      <c r="L59" s="45"/>
-      <c r="M59" s="45"/>
-      <c r="N59" s="46"/>
-      <c r="O59" s="45"/>
-      <c r="P59" s="47"/>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="59" ht="28.5" customHeight="1" spans="1:39">
+      <c r="A59" s="64"/>
+      <c r="B59" s="65"/>
+      <c r="C59" s="65"/>
+      <c r="D59" s="64"/>
+      <c r="E59" s="66"/>
+      <c r="F59" s="64"/>
+      <c r="G59" s="64"/>
+      <c r="H59" s="67"/>
+      <c r="I59" s="68"/>
+      <c r="J59" s="65"/>
+      <c r="K59" s="64"/>
+      <c r="L59" s="65"/>
+      <c r="M59" s="65"/>
+      <c r="N59" s="69"/>
+      <c r="O59" s="65"/>
+      <c r="P59" s="70"/>
       <c r="Q59" s="63"/>
       <c r="R59" s="63"/>
-      <c r="S59" s="47"/>
-      <c r="T59" s="47"/>
-      <c r="U59" s="32"/>
+      <c r="S59" s="70"/>
+      <c r="T59" s="70"/>
+      <c r="U59" s="72"/>
       <c r="V59" s="48"/>
       <c r="W59" s="48"/>
       <c r="X59" s="48"/>
-      <c r="Y59" s="41"/>
-      <c r="Z59" s="41"/>
-      <c r="AA59" s="49"/>
-      <c r="AB59" s="49"/>
-      <c r="AC59" s="49"/>
-      <c r="AD59" s="49"/>
-      <c r="AE59" s="45"/>
-      <c r="AF59" s="45"/>
-      <c r="AG59" s="50"/>
-      <c r="AH59" s="50"/>
-      <c r="AI59" s="50"/>
-      <c r="AJ59" s="50"/>
-      <c r="AK59" s="50"/>
+      <c r="Y59" s="64"/>
+      <c r="Z59" s="75"/>
+      <c r="AA59" s="73"/>
+      <c r="AB59" s="73"/>
+      <c r="AC59" s="73"/>
+      <c r="AD59" s="73"/>
+      <c r="AE59" s="65"/>
+      <c r="AF59" s="65"/>
+      <c r="AG59" s="74"/>
+      <c r="AH59" s="74"/>
+      <c r="AI59" s="74"/>
+      <c r="AJ59" s="74"/>
+      <c r="AK59" s="74"/>
       <c r="AL59" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM59" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="60" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -4587,10 +4582,10 @@
       <c r="AJ60" s="50"/>
       <c r="AK60" s="50"/>
       <c r="AL60" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM60" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="61" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -4632,10 +4627,10 @@
       <c r="AJ61" s="50"/>
       <c r="AK61" s="50"/>
       <c r="AL61" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM61" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="62" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -4677,10 +4672,10 @@
       <c r="AJ62" s="50"/>
       <c r="AK62" s="50"/>
       <c r="AL62" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM62" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="63" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -4722,10 +4717,10 @@
       <c r="AJ63" s="50"/>
       <c r="AK63" s="50"/>
       <c r="AL63" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM63" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="64" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -4767,10 +4762,10 @@
       <c r="AJ64" s="50"/>
       <c r="AK64" s="50"/>
       <c r="AL64" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM64" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="65" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -4812,10 +4807,10 @@
       <c r="AJ65" s="50"/>
       <c r="AK65" s="50"/>
       <c r="AL65" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM65" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="66" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -4857,10 +4852,10 @@
       <c r="AJ66" s="50"/>
       <c r="AK66" s="50"/>
       <c r="AL66" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM66" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="67" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -4902,10 +4897,10 @@
       <c r="AJ67" s="50"/>
       <c r="AK67" s="50"/>
       <c r="AL67" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM67" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="68" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -4947,10 +4942,10 @@
       <c r="AJ68" s="50"/>
       <c r="AK68" s="50"/>
       <c r="AL68" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM68" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="69" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -4992,10 +4987,10 @@
       <c r="AJ69" s="50"/>
       <c r="AK69" s="50"/>
       <c r="AL69" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM69" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="70" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5037,10 +5032,10 @@
       <c r="AJ70" s="50"/>
       <c r="AK70" s="50"/>
       <c r="AL70" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM70" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="71" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5082,10 +5077,10 @@
       <c r="AJ71" s="50"/>
       <c r="AK71" s="50"/>
       <c r="AL71" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM71" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="72" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5127,10 +5122,10 @@
       <c r="AJ72" s="50"/>
       <c r="AK72" s="50"/>
       <c r="AL72" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM72" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="73" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5172,10 +5167,10 @@
       <c r="AJ73" s="50"/>
       <c r="AK73" s="50"/>
       <c r="AL73" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM73" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="74" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5217,10 +5212,10 @@
       <c r="AJ74" s="50"/>
       <c r="AK74" s="50"/>
       <c r="AL74" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM74" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="75" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5262,10 +5257,10 @@
       <c r="AJ75" s="50"/>
       <c r="AK75" s="50"/>
       <c r="AL75" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM75" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="76" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5307,10 +5302,10 @@
       <c r="AJ76" s="50"/>
       <c r="AK76" s="50"/>
       <c r="AL76" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM76" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="77" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5352,10 +5347,10 @@
       <c r="AJ77" s="50"/>
       <c r="AK77" s="50"/>
       <c r="AL77" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM77" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="78" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5397,10 +5392,10 @@
       <c r="AJ78" s="50"/>
       <c r="AK78" s="50"/>
       <c r="AL78" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM78" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="79" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5442,10 +5437,10 @@
       <c r="AJ79" s="50"/>
       <c r="AK79" s="50"/>
       <c r="AL79" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM79" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="80" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5487,10 +5482,10 @@
       <c r="AJ80" s="50"/>
       <c r="AK80" s="50"/>
       <c r="AL80" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM80" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="81" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5532,10 +5527,10 @@
       <c r="AJ81" s="50"/>
       <c r="AK81" s="50"/>
       <c r="AL81" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM81" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="82" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5577,10 +5572,10 @@
       <c r="AJ82" s="50"/>
       <c r="AK82" s="50"/>
       <c r="AL82" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM82" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="83" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5622,10 +5617,10 @@
       <c r="AJ83" s="50"/>
       <c r="AK83" s="50"/>
       <c r="AL83" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM83" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="84" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5667,10 +5662,10 @@
       <c r="AJ84" s="50"/>
       <c r="AK84" s="50"/>
       <c r="AL84" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM84" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="85" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5712,10 +5707,10 @@
       <c r="AJ85" s="50"/>
       <c r="AK85" s="50"/>
       <c r="AL85" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM85" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="86" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5757,10 +5752,10 @@
       <c r="AJ86" s="50"/>
       <c r="AK86" s="50"/>
       <c r="AL86" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM86" s="39" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="87" s="2" customFormat="1" customHeight="1" spans="1:39">
@@ -5802,145 +5797,145 @@
       <c r="AJ87" s="50"/>
       <c r="AK87" s="50"/>
       <c r="AL87" s="39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM87" s="39" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="88" s="2" customFormat="1" customHeight="1" spans="1:39">
+      <c r="A88" s="41"/>
+      <c r="B88" s="45"/>
+      <c r="C88" s="45"/>
+      <c r="D88" s="41"/>
+      <c r="E88" s="42"/>
+      <c r="F88" s="41"/>
+      <c r="G88" s="41"/>
+      <c r="H88" s="43"/>
+      <c r="I88" s="44"/>
+      <c r="J88" s="45"/>
+      <c r="K88" s="41"/>
+      <c r="L88" s="45"/>
+      <c r="M88" s="45"/>
+      <c r="N88" s="46"/>
+      <c r="O88" s="45"/>
+      <c r="P88" s="47"/>
+      <c r="Q88" s="63"/>
+      <c r="R88" s="63"/>
+      <c r="S88" s="47"/>
+      <c r="T88" s="47"/>
+      <c r="U88" s="32"/>
+      <c r="V88" s="48"/>
+      <c r="W88" s="48"/>
+      <c r="X88" s="48"/>
+      <c r="Y88" s="41"/>
+      <c r="Z88" s="41"/>
+      <c r="AA88" s="49"/>
+      <c r="AB88" s="49"/>
+      <c r="AC88" s="49"/>
+      <c r="AD88" s="49"/>
+      <c r="AE88" s="45"/>
+      <c r="AF88" s="45"/>
+      <c r="AG88" s="50"/>
+      <c r="AH88" s="50"/>
+      <c r="AI88" s="50"/>
+      <c r="AJ88" s="50"/>
+      <c r="AK88" s="50"/>
+      <c r="AL88" s="39" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="88" s="4" customFormat="1" customHeight="1" spans="1:39">
-      <c r="A88" s="76"/>
-      <c r="B88" s="77"/>
-      <c r="C88" s="77"/>
-      <c r="D88" s="76"/>
-      <c r="E88" s="78"/>
-      <c r="F88" s="76"/>
-      <c r="G88" s="76"/>
-      <c r="H88" s="79"/>
-      <c r="I88" s="80"/>
-      <c r="J88" s="77"/>
-      <c r="K88" s="76"/>
-      <c r="L88" s="77"/>
-      <c r="M88" s="77"/>
-      <c r="N88" s="81"/>
-      <c r="O88" s="77"/>
-      <c r="P88" s="82"/>
-      <c r="Q88" s="83"/>
-      <c r="R88" s="83"/>
-      <c r="S88" s="84"/>
-      <c r="T88" s="84"/>
-      <c r="U88" s="85"/>
-      <c r="V88" s="86"/>
-      <c r="W88" s="86"/>
-      <c r="X88" s="86"/>
-      <c r="Y88" s="76"/>
-      <c r="Z88" s="76"/>
-      <c r="AA88" s="87"/>
-      <c r="AB88" s="87"/>
-      <c r="AC88" s="87"/>
-      <c r="AD88" s="87"/>
-      <c r="AE88" s="77"/>
-      <c r="AF88" s="77"/>
-      <c r="AG88" s="88"/>
-      <c r="AH88" s="88"/>
-      <c r="AI88" s="88"/>
-      <c r="AJ88" s="88"/>
-      <c r="AK88" s="88"/>
-      <c r="AL88" s="89" t="s">
-        <v>64</v>
-      </c>
-      <c r="AM88" s="89" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="89" customHeight="1" spans="1:39">
-      <c r="A89" s="64"/>
-      <c r="B89" s="65"/>
-      <c r="C89" s="65"/>
-      <c r="D89" s="64"/>
-      <c r="E89" s="66"/>
-      <c r="F89" s="64"/>
-      <c r="G89" s="64"/>
-      <c r="H89" s="67"/>
-      <c r="I89" s="68"/>
-      <c r="J89" s="65"/>
-      <c r="K89" s="64"/>
-      <c r="L89" s="65"/>
-      <c r="M89" s="65"/>
-      <c r="N89" s="69"/>
-      <c r="O89" s="65"/>
-      <c r="P89" s="70"/>
+      <c r="AM88" s="39" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="89" s="2" customFormat="1" customHeight="1" spans="1:39">
+      <c r="A89" s="41"/>
+      <c r="B89" s="45"/>
+      <c r="C89" s="45"/>
+      <c r="D89" s="41"/>
+      <c r="E89" s="42"/>
+      <c r="F89" s="41"/>
+      <c r="G89" s="41"/>
+      <c r="H89" s="43"/>
+      <c r="I89" s="44"/>
+      <c r="J89" s="45"/>
+      <c r="K89" s="41"/>
+      <c r="L89" s="45"/>
+      <c r="M89" s="45"/>
+      <c r="N89" s="46"/>
+      <c r="O89" s="45"/>
+      <c r="P89" s="47"/>
       <c r="Q89" s="63"/>
       <c r="R89" s="63"/>
       <c r="S89" s="47"/>
       <c r="T89" s="47"/>
-      <c r="U89" s="72"/>
+      <c r="U89" s="32"/>
       <c r="V89" s="48"/>
       <c r="W89" s="48"/>
       <c r="X89" s="48"/>
-      <c r="Y89" s="64"/>
-      <c r="Z89" s="64"/>
-      <c r="AA89" s="73"/>
-      <c r="AB89" s="73"/>
-      <c r="AC89" s="73"/>
-      <c r="AD89" s="73"/>
-      <c r="AE89" s="65"/>
-      <c r="AF89" s="65"/>
-      <c r="AG89" s="74"/>
-      <c r="AH89" s="74"/>
-      <c r="AI89" s="74"/>
-      <c r="AJ89" s="74"/>
-      <c r="AK89" s="74"/>
-      <c r="AL89" s="90" t="s">
-        <v>64</v>
-      </c>
-      <c r="AM89" s="91" t="s">
+      <c r="Y89" s="41"/>
+      <c r="Z89" s="41"/>
+      <c r="AA89" s="49"/>
+      <c r="AB89" s="49"/>
+      <c r="AC89" s="49"/>
+      <c r="AD89" s="49"/>
+      <c r="AE89" s="45"/>
+      <c r="AF89" s="45"/>
+      <c r="AG89" s="50"/>
+      <c r="AH89" s="50"/>
+      <c r="AI89" s="50"/>
+      <c r="AJ89" s="50"/>
+      <c r="AK89" s="50"/>
+      <c r="AL89" s="39" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="90" customHeight="1" spans="1:39">
-      <c r="A90" s="64"/>
-      <c r="B90" s="65"/>
-      <c r="C90" s="65"/>
-      <c r="D90" s="64"/>
-      <c r="E90" s="66"/>
-      <c r="F90" s="64"/>
-      <c r="G90" s="64"/>
-      <c r="H90" s="67"/>
-      <c r="I90" s="68"/>
-      <c r="J90" s="65"/>
-      <c r="K90" s="64"/>
-      <c r="L90" s="65"/>
-      <c r="M90" s="65"/>
-      <c r="N90" s="69"/>
-      <c r="O90" s="65"/>
-      <c r="P90" s="70"/>
-      <c r="Q90" s="63"/>
-      <c r="R90" s="63"/>
-      <c r="S90" s="70"/>
-      <c r="T90" s="70"/>
-      <c r="U90" s="72"/>
-      <c r="V90" s="48"/>
-      <c r="W90" s="48"/>
-      <c r="X90" s="48"/>
-      <c r="Y90" s="64"/>
-      <c r="Z90" s="64"/>
-      <c r="AA90" s="73"/>
-      <c r="AB90" s="73"/>
-      <c r="AC90" s="73"/>
-      <c r="AD90" s="73"/>
-      <c r="AE90" s="65"/>
-      <c r="AF90" s="65"/>
-      <c r="AG90" s="74"/>
-      <c r="AH90" s="74"/>
-      <c r="AI90" s="74"/>
-      <c r="AJ90" s="74"/>
-      <c r="AK90" s="74"/>
-      <c r="AL90" s="90" t="s">
-        <v>64</v>
-      </c>
-      <c r="AM90" s="91" t="s">
+      <c r="AM89" s="39" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="90" s="4" customFormat="1" customHeight="1" spans="1:39">
+      <c r="A90" s="76"/>
+      <c r="B90" s="77"/>
+      <c r="C90" s="77"/>
+      <c r="D90" s="76"/>
+      <c r="E90" s="78"/>
+      <c r="F90" s="76"/>
+      <c r="G90" s="76"/>
+      <c r="H90" s="79"/>
+      <c r="I90" s="80"/>
+      <c r="J90" s="77"/>
+      <c r="K90" s="76"/>
+      <c r="L90" s="77"/>
+      <c r="M90" s="77"/>
+      <c r="N90" s="81"/>
+      <c r="O90" s="77"/>
+      <c r="P90" s="82"/>
+      <c r="Q90" s="83"/>
+      <c r="R90" s="83"/>
+      <c r="S90" s="84"/>
+      <c r="T90" s="84"/>
+      <c r="U90" s="85"/>
+      <c r="V90" s="86"/>
+      <c r="W90" s="86"/>
+      <c r="X90" s="86"/>
+      <c r="Y90" s="76"/>
+      <c r="Z90" s="76"/>
+      <c r="AA90" s="87"/>
+      <c r="AB90" s="87"/>
+      <c r="AC90" s="87"/>
+      <c r="AD90" s="87"/>
+      <c r="AE90" s="77"/>
+      <c r="AF90" s="77"/>
+      <c r="AG90" s="88"/>
+      <c r="AH90" s="88"/>
+      <c r="AI90" s="88"/>
+      <c r="AJ90" s="88"/>
+      <c r="AK90" s="88"/>
+      <c r="AL90" s="89" t="s">
         <v>65</v>
+      </c>
+      <c r="AM90" s="89" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="91" customHeight="1" spans="1:39">
@@ -5962,8 +5957,8 @@
       <c r="P91" s="70"/>
       <c r="Q91" s="63"/>
       <c r="R91" s="63"/>
-      <c r="S91" s="70"/>
-      <c r="T91" s="70"/>
+      <c r="S91" s="47"/>
+      <c r="T91" s="47"/>
       <c r="U91" s="72"/>
       <c r="V91" s="48"/>
       <c r="W91" s="48"/>
@@ -5982,10 +5977,10 @@
       <c r="AJ91" s="74"/>
       <c r="AK91" s="74"/>
       <c r="AL91" s="90" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM91" s="91" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="92" customHeight="1" spans="1:39">
@@ -6027,10 +6022,10 @@
       <c r="AJ92" s="74"/>
       <c r="AK92" s="74"/>
       <c r="AL92" s="90" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM92" s="91" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="93" customHeight="1" spans="1:39">
@@ -6038,26 +6033,26 @@
       <c r="B93" s="65"/>
       <c r="C93" s="65"/>
       <c r="D93" s="64"/>
-      <c r="E93" s="75"/>
+      <c r="E93" s="66"/>
       <c r="F93" s="64"/>
       <c r="G93" s="64"/>
-      <c r="H93" s="92"/>
+      <c r="H93" s="67"/>
       <c r="I93" s="68"/>
       <c r="J93" s="65"/>
       <c r="K93" s="64"/>
       <c r="L93" s="65"/>
       <c r="M93" s="65"/>
-      <c r="N93" s="93"/>
+      <c r="N93" s="69"/>
       <c r="O93" s="65"/>
-      <c r="P93" s="94"/>
-      <c r="Q93" s="95"/>
-      <c r="R93" s="95"/>
-      <c r="S93" s="94"/>
-      <c r="T93" s="94"/>
-      <c r="U93" s="96"/>
-      <c r="V93" s="97"/>
-      <c r="W93" s="97"/>
-      <c r="X93" s="97"/>
+      <c r="P93" s="70"/>
+      <c r="Q93" s="63"/>
+      <c r="R93" s="63"/>
+      <c r="S93" s="70"/>
+      <c r="T93" s="70"/>
+      <c r="U93" s="72"/>
+      <c r="V93" s="48"/>
+      <c r="W93" s="48"/>
+      <c r="X93" s="48"/>
       <c r="Y93" s="64"/>
       <c r="Z93" s="64"/>
       <c r="AA93" s="73"/>
@@ -6072,57 +6067,55 @@
       <c r="AJ93" s="74"/>
       <c r="AK93" s="74"/>
       <c r="AL93" s="90" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM93" s="91" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="94" customHeight="1" spans="1:39">
+      <c r="A94" s="64"/>
+      <c r="B94" s="65"/>
+      <c r="C94" s="65"/>
+      <c r="D94" s="64"/>
+      <c r="E94" s="66"/>
+      <c r="F94" s="64"/>
+      <c r="G94" s="64"/>
+      <c r="H94" s="67"/>
+      <c r="I94" s="68"/>
+      <c r="J94" s="65"/>
+      <c r="K94" s="64"/>
+      <c r="L94" s="65"/>
+      <c r="M94" s="65"/>
+      <c r="N94" s="69"/>
+      <c r="O94" s="65"/>
+      <c r="P94" s="70"/>
+      <c r="Q94" s="63"/>
+      <c r="R94" s="63"/>
+      <c r="S94" s="70"/>
+      <c r="T94" s="70"/>
+      <c r="U94" s="72"/>
+      <c r="V94" s="48"/>
+      <c r="W94" s="48"/>
+      <c r="X94" s="48"/>
+      <c r="Y94" s="64"/>
+      <c r="Z94" s="64"/>
+      <c r="AA94" s="73"/>
+      <c r="AB94" s="73"/>
+      <c r="AC94" s="73"/>
+      <c r="AD94" s="73"/>
+      <c r="AE94" s="65"/>
+      <c r="AF94" s="65"/>
+      <c r="AG94" s="74"/>
+      <c r="AH94" s="74"/>
+      <c r="AI94" s="74"/>
+      <c r="AJ94" s="74"/>
+      <c r="AK94" s="74"/>
+      <c r="AL94" s="90" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="94" s="4" customFormat="1" customHeight="1" spans="1:39">
-      <c r="A94" s="76"/>
-      <c r="B94" s="77"/>
-      <c r="C94" s="77"/>
-      <c r="D94" s="76"/>
-      <c r="E94" s="78"/>
-      <c r="F94" s="76"/>
-      <c r="G94" s="76"/>
-      <c r="H94" s="79"/>
-      <c r="I94" s="80"/>
-      <c r="J94" s="77"/>
-      <c r="K94" s="76"/>
-      <c r="L94" s="77"/>
-      <c r="M94" s="77"/>
-      <c r="N94" s="81"/>
-      <c r="O94" s="77"/>
-      <c r="P94" s="82"/>
-      <c r="Q94" s="83"/>
-      <c r="R94" s="83"/>
-      <c r="S94" s="82"/>
-      <c r="T94" s="82"/>
-      <c r="U94" s="85"/>
-      <c r="V94" s="86"/>
-      <c r="W94" s="86"/>
-      <c r="X94" s="86"/>
-      <c r="Y94" s="76"/>
-      <c r="Z94" s="76"/>
-      <c r="AA94" s="87"/>
-      <c r="AB94" s="87"/>
-      <c r="AC94" s="87"/>
-      <c r="AD94" s="87"/>
-      <c r="AE94" s="110" t="s">
-        <v>68</v>
-      </c>
-      <c r="AF94" s="77"/>
-      <c r="AG94" s="88"/>
-      <c r="AH94" s="88"/>
-      <c r="AI94" s="88"/>
-      <c r="AJ94" s="88"/>
-      <c r="AK94" s="88"/>
-      <c r="AL94" s="98" t="s">
-        <v>64</v>
-      </c>
-      <c r="AM94" s="99" t="s">
-        <v>65</v>
+      <c r="AM94" s="91" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="95" customHeight="1" spans="1:39">
@@ -6130,26 +6123,26 @@
       <c r="B95" s="65"/>
       <c r="C95" s="65"/>
       <c r="D95" s="64"/>
-      <c r="E95" s="66"/>
+      <c r="E95" s="75"/>
       <c r="F95" s="64"/>
       <c r="G95" s="64"/>
-      <c r="H95" s="67"/>
+      <c r="H95" s="92"/>
       <c r="I95" s="68"/>
       <c r="J95" s="65"/>
       <c r="K95" s="64"/>
       <c r="L95" s="65"/>
       <c r="M95" s="65"/>
-      <c r="N95" s="69"/>
+      <c r="N95" s="93"/>
       <c r="O95" s="65"/>
-      <c r="P95" s="70"/>
-      <c r="Q95" s="63"/>
-      <c r="R95" s="63"/>
-      <c r="S95" s="70"/>
-      <c r="T95" s="70"/>
-      <c r="U95" s="72"/>
-      <c r="V95" s="48"/>
-      <c r="W95" s="48"/>
-      <c r="X95" s="48"/>
+      <c r="P95" s="94"/>
+      <c r="Q95" s="95"/>
+      <c r="R95" s="95"/>
+      <c r="S95" s="94"/>
+      <c r="T95" s="94"/>
+      <c r="U95" s="96"/>
+      <c r="V95" s="97"/>
+      <c r="W95" s="97"/>
+      <c r="X95" s="97"/>
       <c r="Y95" s="64"/>
       <c r="Z95" s="64"/>
       <c r="AA95" s="73"/>
@@ -6164,55 +6157,57 @@
       <c r="AJ95" s="74"/>
       <c r="AK95" s="74"/>
       <c r="AL95" s="90" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM95" s="91" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="96" s="4" customFormat="1" customHeight="1" spans="1:39">
+      <c r="A96" s="76"/>
+      <c r="B96" s="77"/>
+      <c r="C96" s="77"/>
+      <c r="D96" s="76"/>
+      <c r="E96" s="78"/>
+      <c r="F96" s="76"/>
+      <c r="G96" s="76"/>
+      <c r="H96" s="79"/>
+      <c r="I96" s="80"/>
+      <c r="J96" s="77"/>
+      <c r="K96" s="76"/>
+      <c r="L96" s="77"/>
+      <c r="M96" s="77"/>
+      <c r="N96" s="81"/>
+      <c r="O96" s="77"/>
+      <c r="P96" s="82"/>
+      <c r="Q96" s="83"/>
+      <c r="R96" s="83"/>
+      <c r="S96" s="82"/>
+      <c r="T96" s="82"/>
+      <c r="U96" s="85"/>
+      <c r="V96" s="86"/>
+      <c r="W96" s="86"/>
+      <c r="X96" s="86"/>
+      <c r="Y96" s="76"/>
+      <c r="Z96" s="76"/>
+      <c r="AA96" s="87"/>
+      <c r="AB96" s="87"/>
+      <c r="AC96" s="87"/>
+      <c r="AD96" s="87"/>
+      <c r="AE96" s="110" t="s">
+        <v>69</v>
+      </c>
+      <c r="AF96" s="77"/>
+      <c r="AG96" s="88"/>
+      <c r="AH96" s="88"/>
+      <c r="AI96" s="88"/>
+      <c r="AJ96" s="88"/>
+      <c r="AK96" s="88"/>
+      <c r="AL96" s="98" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="96" customHeight="1" spans="1:39">
-      <c r="A96" s="64"/>
-      <c r="B96" s="65"/>
-      <c r="C96" s="65"/>
-      <c r="D96" s="64"/>
-      <c r="E96" s="66"/>
-      <c r="F96" s="64"/>
-      <c r="G96" s="64"/>
-      <c r="H96" s="67"/>
-      <c r="I96" s="68"/>
-      <c r="J96" s="65"/>
-      <c r="K96" s="64"/>
-      <c r="L96" s="65"/>
-      <c r="M96" s="65"/>
-      <c r="N96" s="69"/>
-      <c r="O96" s="65"/>
-      <c r="P96" s="70"/>
-      <c r="Q96" s="63"/>
-      <c r="R96" s="63"/>
-      <c r="S96" s="70"/>
-      <c r="T96" s="70"/>
-      <c r="U96" s="72"/>
-      <c r="V96" s="48"/>
-      <c r="W96" s="48"/>
-      <c r="X96" s="48"/>
-      <c r="Y96" s="64"/>
-      <c r="Z96" s="64"/>
-      <c r="AA96" s="73"/>
-      <c r="AB96" s="73"/>
-      <c r="AC96" s="73"/>
-      <c r="AD96" s="73"/>
-      <c r="AE96" s="65"/>
-      <c r="AF96" s="65"/>
-      <c r="AG96" s="74"/>
-      <c r="AH96" s="74"/>
-      <c r="AI96" s="74"/>
-      <c r="AJ96" s="74"/>
-      <c r="AK96" s="74"/>
-      <c r="AL96" s="90" t="s">
-        <v>64</v>
-      </c>
-      <c r="AM96" s="91" t="s">
-        <v>65</v>
+      <c r="AM96" s="99" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="97" customHeight="1" spans="1:39">
@@ -6232,8 +6227,8 @@
       <c r="N97" s="69"/>
       <c r="O97" s="65"/>
       <c r="P97" s="70"/>
-      <c r="Q97" s="71"/>
-      <c r="R97" s="70"/>
+      <c r="Q97" s="63"/>
+      <c r="R97" s="63"/>
       <c r="S97" s="70"/>
       <c r="T97" s="70"/>
       <c r="U97" s="72"/>
@@ -6254,10 +6249,10 @@
       <c r="AJ97" s="74"/>
       <c r="AK97" s="74"/>
       <c r="AL97" s="90" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM97" s="91" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="98" customHeight="1" spans="1:39">
@@ -6277,8 +6272,8 @@
       <c r="N98" s="69"/>
       <c r="O98" s="65"/>
       <c r="P98" s="70"/>
-      <c r="Q98" s="71"/>
-      <c r="R98" s="70"/>
+      <c r="Q98" s="63"/>
+      <c r="R98" s="63"/>
       <c r="S98" s="70"/>
       <c r="T98" s="70"/>
       <c r="U98" s="72"/>
@@ -6299,10 +6294,10 @@
       <c r="AJ98" s="74"/>
       <c r="AK98" s="74"/>
       <c r="AL98" s="90" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM98" s="91" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="99" customHeight="1" spans="1:39">
@@ -6344,10 +6339,10 @@
       <c r="AJ99" s="74"/>
       <c r="AK99" s="74"/>
       <c r="AL99" s="90" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM99" s="91" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="100" customHeight="1" spans="1:39">
@@ -6389,20 +6384,20 @@
       <c r="AJ100" s="74"/>
       <c r="AK100" s="74"/>
       <c r="AL100" s="90" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM100" s="91" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="101" s="5" customFormat="1" customHeight="1" spans="1:39">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="101" customHeight="1" spans="1:39">
       <c r="A101" s="64"/>
       <c r="B101" s="65"/>
       <c r="C101" s="65"/>
       <c r="D101" s="64"/>
       <c r="E101" s="66"/>
-      <c r="F101" s="41"/>
-      <c r="G101" s="41"/>
+      <c r="F101" s="64"/>
+      <c r="G101" s="64"/>
       <c r="H101" s="67"/>
       <c r="I101" s="68"/>
       <c r="J101" s="65"/>
@@ -6434,10 +6429,10 @@
       <c r="AJ101" s="74"/>
       <c r="AK101" s="74"/>
       <c r="AL101" s="90" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM101" s="91" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="102" customHeight="1" spans="1:39">
@@ -6457,8 +6452,8 @@
       <c r="N102" s="69"/>
       <c r="O102" s="65"/>
       <c r="P102" s="70"/>
-      <c r="Q102" s="63"/>
-      <c r="R102" s="63"/>
+      <c r="Q102" s="71"/>
+      <c r="R102" s="70"/>
       <c r="S102" s="70"/>
       <c r="T102" s="70"/>
       <c r="U102" s="72"/>
@@ -6479,13 +6474,13 @@
       <c r="AJ102" s="74"/>
       <c r="AK102" s="74"/>
       <c r="AL102" s="90" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM102" s="91" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="103" customHeight="1" spans="1:39">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="103" s="5" customFormat="1" customHeight="1" spans="1:39">
       <c r="A103" s="64"/>
       <c r="B103" s="65"/>
       <c r="C103" s="65"/>
@@ -6524,10 +6519,10 @@
       <c r="AJ103" s="74"/>
       <c r="AK103" s="74"/>
       <c r="AL103" s="90" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM103" s="91" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="104" customHeight="1" spans="1:39">
@@ -6569,79 +6564,101 @@
       <c r="AJ104" s="74"/>
       <c r="AK104" s="74"/>
       <c r="AL104" s="90" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AM104" s="91" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="105" customHeight="1" spans="1:39">
+      <c r="A105" s="64"/>
+      <c r="B105" s="65"/>
+      <c r="C105" s="65"/>
+      <c r="D105" s="64"/>
+      <c r="E105" s="66"/>
+      <c r="F105" s="41"/>
+      <c r="G105" s="41"/>
+      <c r="H105" s="67"/>
+      <c r="I105" s="68"/>
+      <c r="J105" s="65"/>
+      <c r="K105" s="64"/>
+      <c r="L105" s="65"/>
+      <c r="M105" s="65"/>
+      <c r="N105" s="69"/>
+      <c r="O105" s="65"/>
+      <c r="P105" s="70"/>
+      <c r="Q105" s="71"/>
+      <c r="R105" s="70"/>
+      <c r="S105" s="70"/>
+      <c r="T105" s="70"/>
+      <c r="U105" s="72"/>
+      <c r="V105" s="48"/>
+      <c r="W105" s="48"/>
+      <c r="X105" s="48"/>
+      <c r="Y105" s="64"/>
+      <c r="Z105" s="64"/>
+      <c r="AA105" s="73"/>
+      <c r="AB105" s="73"/>
+      <c r="AC105" s="73"/>
+      <c r="AD105" s="73"/>
+      <c r="AE105" s="65"/>
+      <c r="AF105" s="65"/>
+      <c r="AG105" s="74"/>
+      <c r="AH105" s="74"/>
+      <c r="AI105" s="74"/>
+      <c r="AJ105" s="74"/>
+      <c r="AK105" s="74"/>
+      <c r="AL105" s="90" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="105" customHeight="1" spans="1:39">
-      <c r="A105" s="6"/>
-      <c r="B105" s="6"/>
-      <c r="C105" s="6"/>
-      <c r="D105" s="6"/>
-      <c r="E105" s="6"/>
-      <c r="F105" s="6"/>
-      <c r="G105" s="6"/>
-      <c r="H105" s="6"/>
-      <c r="I105" s="6"/>
-      <c r="J105" s="100"/>
-      <c r="K105" s="6"/>
-      <c r="L105" s="100"/>
-      <c r="M105" s="100"/>
-      <c r="N105" s="6"/>
-      <c r="O105" s="100"/>
-      <c r="P105" s="6"/>
-      <c r="Q105" s="6"/>
-      <c r="R105" s="6"/>
-      <c r="S105" s="6"/>
-      <c r="T105" s="6"/>
-      <c r="U105" s="6"/>
-      <c r="V105" s="6"/>
-      <c r="W105" s="6"/>
-      <c r="X105" s="6"/>
-      <c r="Y105" s="6"/>
-      <c r="Z105" s="6"/>
-      <c r="AA105" s="6"/>
-      <c r="AB105" s="6"/>
-      <c r="AC105" s="6"/>
-      <c r="AD105" s="6"/>
-      <c r="AE105" s="6"/>
-      <c r="AF105" s="6"/>
+      <c r="AM105" s="91" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="106" customHeight="1" spans="1:39">
-      <c r="A106" s="6"/>
-      <c r="B106" s="6"/>
-      <c r="C106" s="6"/>
-      <c r="D106" s="6"/>
-      <c r="E106" s="6"/>
-      <c r="F106" s="6"/>
-      <c r="G106" s="6"/>
-      <c r="H106" s="6"/>
-      <c r="I106" s="6"/>
-      <c r="J106" s="100"/>
-      <c r="K106" s="6"/>
-      <c r="L106" s="100"/>
-      <c r="M106" s="100"/>
-      <c r="N106" s="6"/>
-      <c r="O106" s="100"/>
-      <c r="P106" s="6"/>
-      <c r="Q106" s="6"/>
-      <c r="R106" s="6"/>
-      <c r="S106" s="6"/>
-      <c r="T106" s="6"/>
-      <c r="U106" s="6"/>
-      <c r="V106" s="6"/>
-      <c r="W106" s="6"/>
-      <c r="X106" s="6"/>
-      <c r="Y106" s="6"/>
-      <c r="Z106" s="6"/>
-      <c r="AA106" s="6"/>
-      <c r="AB106" s="6"/>
-      <c r="AC106" s="6"/>
-      <c r="AD106" s="6"/>
-      <c r="AE106" s="6"/>
-      <c r="AF106" s="6"/>
+      <c r="A106" s="64"/>
+      <c r="B106" s="65"/>
+      <c r="C106" s="65"/>
+      <c r="D106" s="64"/>
+      <c r="E106" s="66"/>
+      <c r="F106" s="64"/>
+      <c r="G106" s="64"/>
+      <c r="H106" s="67"/>
+      <c r="I106" s="68"/>
+      <c r="J106" s="65"/>
+      <c r="K106" s="64"/>
+      <c r="L106" s="65"/>
+      <c r="M106" s="65"/>
+      <c r="N106" s="69"/>
+      <c r="O106" s="65"/>
+      <c r="P106" s="70"/>
+      <c r="Q106" s="63"/>
+      <c r="R106" s="63"/>
+      <c r="S106" s="70"/>
+      <c r="T106" s="70"/>
+      <c r="U106" s="72"/>
+      <c r="V106" s="48"/>
+      <c r="W106" s="48"/>
+      <c r="X106" s="48"/>
+      <c r="Y106" s="64"/>
+      <c r="Z106" s="64"/>
+      <c r="AA106" s="73"/>
+      <c r="AB106" s="73"/>
+      <c r="AC106" s="73"/>
+      <c r="AD106" s="73"/>
+      <c r="AE106" s="65"/>
+      <c r="AF106" s="65"/>
+      <c r="AG106" s="74"/>
+      <c r="AH106" s="74"/>
+      <c r="AI106" s="74"/>
+      <c r="AJ106" s="74"/>
+      <c r="AK106" s="74"/>
+      <c r="AL106" s="90" t="s">
+        <v>65</v>
+      </c>
+      <c r="AM106" s="91" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="107" customHeight="1" spans="1:39">
       <c r="A107" s="6"/>
@@ -6779,17 +6796,73 @@
       <c r="AE110" s="6"/>
       <c r="AF110" s="6"/>
     </row>
-    <row r="111" s="6" customFormat="1" customHeight="1" spans="1:39">
+    <row r="111" customHeight="1" spans="1:39">
+      <c r="A111" s="6"/>
+      <c r="B111" s="6"/>
+      <c r="C111" s="6"/>
+      <c r="D111" s="6"/>
+      <c r="E111" s="6"/>
+      <c r="F111" s="6"/>
+      <c r="G111" s="6"/>
+      <c r="H111" s="6"/>
+      <c r="I111" s="6"/>
       <c r="J111" s="100"/>
+      <c r="K111" s="6"/>
       <c r="L111" s="100"/>
       <c r="M111" s="100"/>
+      <c r="N111" s="6"/>
       <c r="O111" s="100"/>
-    </row>
-    <row r="112" s="6" customFormat="1" customHeight="1" spans="1:39">
+      <c r="P111" s="6"/>
+      <c r="Q111" s="6"/>
+      <c r="R111" s="6"/>
+      <c r="S111" s="6"/>
+      <c r="T111" s="6"/>
+      <c r="U111" s="6"/>
+      <c r="V111" s="6"/>
+      <c r="W111" s="6"/>
+      <c r="X111" s="6"/>
+      <c r="Y111" s="6"/>
+      <c r="Z111" s="6"/>
+      <c r="AA111" s="6"/>
+      <c r="AB111" s="6"/>
+      <c r="AC111" s="6"/>
+      <c r="AD111" s="6"/>
+      <c r="AE111" s="6"/>
+      <c r="AF111" s="6"/>
+    </row>
+    <row r="112" customHeight="1" spans="1:39">
+      <c r="A112" s="6"/>
+      <c r="B112" s="6"/>
+      <c r="C112" s="6"/>
+      <c r="D112" s="6"/>
+      <c r="E112" s="6"/>
+      <c r="F112" s="6"/>
+      <c r="G112" s="6"/>
+      <c r="H112" s="6"/>
+      <c r="I112" s="6"/>
       <c r="J112" s="100"/>
+      <c r="K112" s="6"/>
       <c r="L112" s="100"/>
       <c r="M112" s="100"/>
+      <c r="N112" s="6"/>
       <c r="O112" s="100"/>
+      <c r="P112" s="6"/>
+      <c r="Q112" s="6"/>
+      <c r="R112" s="6"/>
+      <c r="S112" s="6"/>
+      <c r="T112" s="6"/>
+      <c r="U112" s="6"/>
+      <c r="V112" s="6"/>
+      <c r="W112" s="6"/>
+      <c r="X112" s="6"/>
+      <c r="Y112" s="6"/>
+      <c r="Z112" s="6"/>
+      <c r="AA112" s="6"/>
+      <c r="AB112" s="6"/>
+      <c r="AC112" s="6"/>
+      <c r="AD112" s="6"/>
+      <c r="AE112" s="6"/>
+      <c r="AF112" s="6"/>
     </row>
     <row r="113" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J113" s="100"/>
@@ -6971,7 +7044,7 @@
       <c r="M142" s="100"/>
       <c r="O142" s="100"/>
     </row>
-    <row r="143" s="6" customFormat="1" ht="18.75" customHeight="1" spans="10:15">
+    <row r="143" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J143" s="100"/>
       <c r="L143" s="100"/>
       <c r="M143" s="100"/>
@@ -6983,7 +7056,7 @@
       <c r="M144" s="100"/>
       <c r="O144" s="100"/>
     </row>
-    <row r="145" s="6" customFormat="1" customHeight="1" spans="10:15">
+    <row r="145" s="6" customFormat="1" ht="18.75" customHeight="1" spans="10:15">
       <c r="J145" s="100"/>
       <c r="L145" s="100"/>
       <c r="M145" s="100"/>
@@ -7241,29 +7314,29 @@
       <c r="M187" s="100"/>
       <c r="O187" s="100"/>
     </row>
-    <row r="188" s="7" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J188" s="101"/>
-      <c r="L188" s="101"/>
-      <c r="M188" s="101"/>
-      <c r="O188" s="101"/>
-    </row>
-    <row r="189" s="4" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J189" s="102"/>
-      <c r="L189" s="102"/>
-      <c r="M189" s="102"/>
-      <c r="O189" s="102"/>
-    </row>
-    <row r="190" s="6" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J190" s="100"/>
-      <c r="L190" s="100"/>
-      <c r="M190" s="100"/>
-      <c r="O190" s="100"/>
-    </row>
-    <row r="191" s="6" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J191" s="100"/>
-      <c r="L191" s="100"/>
-      <c r="M191" s="100"/>
-      <c r="O191" s="100"/>
+    <row r="188" s="6" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J188" s="100"/>
+      <c r="L188" s="100"/>
+      <c r="M188" s="100"/>
+      <c r="O188" s="100"/>
+    </row>
+    <row r="189" s="6" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J189" s="100"/>
+      <c r="L189" s="100"/>
+      <c r="M189" s="100"/>
+      <c r="O189" s="100"/>
+    </row>
+    <row r="190" s="7" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J190" s="101"/>
+      <c r="L190" s="101"/>
+      <c r="M190" s="101"/>
+      <c r="O190" s="101"/>
+    </row>
+    <row r="191" s="4" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J191" s="102"/>
+      <c r="L191" s="102"/>
+      <c r="M191" s="102"/>
+      <c r="O191" s="102"/>
     </row>
     <row r="192" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J192" s="100"/>
@@ -7271,11 +7344,11 @@
       <c r="M192" s="100"/>
       <c r="O192" s="100"/>
     </row>
-    <row r="193" s="8" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J193" s="103"/>
-      <c r="L193" s="103"/>
-      <c r="M193" s="103"/>
-      <c r="O193" s="103"/>
+    <row r="193" s="6" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J193" s="100"/>
+      <c r="L193" s="100"/>
+      <c r="M193" s="100"/>
+      <c r="O193" s="100"/>
     </row>
     <row r="194" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J194" s="100"/>
@@ -7283,11 +7356,11 @@
       <c r="M194" s="100"/>
       <c r="O194" s="100"/>
     </row>
-    <row r="195" s="6" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J195" s="100"/>
-      <c r="L195" s="100"/>
-      <c r="M195" s="100"/>
-      <c r="O195" s="100"/>
+    <row r="195" s="8" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J195" s="103"/>
+      <c r="L195" s="103"/>
+      <c r="M195" s="103"/>
+      <c r="O195" s="103"/>
     </row>
     <row r="196" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J196" s="100"/>
@@ -7295,17 +7368,17 @@
       <c r="M196" s="100"/>
       <c r="O196" s="100"/>
     </row>
-    <row r="197" s="9" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J197" s="104"/>
-      <c r="L197" s="104"/>
-      <c r="M197" s="104"/>
-      <c r="O197" s="104"/>
-    </row>
-    <row r="198" s="9" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J198" s="104"/>
-      <c r="L198" s="104"/>
-      <c r="M198" s="104"/>
-      <c r="O198" s="104"/>
+    <row r="197" s="6" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J197" s="100"/>
+      <c r="L197" s="100"/>
+      <c r="M197" s="100"/>
+      <c r="O197" s="100"/>
+    </row>
+    <row r="198" s="6" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J198" s="100"/>
+      <c r="L198" s="100"/>
+      <c r="M198" s="100"/>
+      <c r="O198" s="100"/>
     </row>
     <row r="199" s="9" customFormat="1" customHeight="1" spans="10:15">
       <c r="J199" s="104"/>
@@ -7535,19 +7608,19 @@
       <c r="M236" s="104"/>
       <c r="O236" s="104"/>
     </row>
-    <row r="237" s="10" customFormat="1" ht="18" customHeight="1" spans="10:15">
-      <c r="J237" s="105"/>
-      <c r="L237" s="105"/>
-      <c r="M237" s="105"/>
-      <c r="O237" s="105"/>
-    </row>
-    <row r="238" s="10" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J238" s="105"/>
-      <c r="L238" s="105"/>
-      <c r="M238" s="105"/>
-      <c r="O238" s="105"/>
-    </row>
-    <row r="239" s="10" customFormat="1" customHeight="1" spans="10:15">
+    <row r="237" s="9" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J237" s="104"/>
+      <c r="L237" s="104"/>
+      <c r="M237" s="104"/>
+      <c r="O237" s="104"/>
+    </row>
+    <row r="238" s="9" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J238" s="104"/>
+      <c r="L238" s="104"/>
+      <c r="M238" s="104"/>
+      <c r="O238" s="104"/>
+    </row>
+    <row r="239" s="10" customFormat="1" ht="18" customHeight="1" spans="10:15">
       <c r="J239" s="105"/>
       <c r="L239" s="105"/>
       <c r="M239" s="105"/>
@@ -7709,17 +7782,17 @@
       <c r="M265" s="105"/>
       <c r="O265" s="105"/>
     </row>
-    <row r="266" s="6" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J266" s="100"/>
-      <c r="L266" s="100"/>
-      <c r="M266" s="100"/>
-      <c r="O266" s="100"/>
-    </row>
-    <row r="267" s="6" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J267" s="100"/>
-      <c r="L267" s="100"/>
-      <c r="M267" s="100"/>
-      <c r="O267" s="100"/>
+    <row r="266" s="10" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J266" s="105"/>
+      <c r="L266" s="105"/>
+      <c r="M266" s="105"/>
+      <c r="O266" s="105"/>
+    </row>
+    <row r="267" s="10" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J267" s="105"/>
+      <c r="L267" s="105"/>
+      <c r="M267" s="105"/>
+      <c r="O267" s="105"/>
     </row>
     <row r="268" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J268" s="100"/>
@@ -7763,29 +7836,29 @@
       <c r="M274" s="100"/>
       <c r="O274" s="100"/>
     </row>
-    <row r="275" s="11" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J275" s="106"/>
-      <c r="L275" s="106"/>
-      <c r="M275" s="106"/>
-      <c r="O275" s="106"/>
-    </row>
-    <row r="276" s="12" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J276" s="107"/>
-      <c r="L276" s="107"/>
-      <c r="M276" s="107"/>
-      <c r="O276" s="107"/>
-    </row>
-    <row r="277" s="6" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J277" s="100"/>
-      <c r="L277" s="100"/>
-      <c r="M277" s="100"/>
-      <c r="O277" s="100"/>
-    </row>
-    <row r="278" s="6" customFormat="1" customHeight="1" spans="10:15">
-      <c r="J278" s="100"/>
-      <c r="L278" s="100"/>
-      <c r="M278" s="100"/>
-      <c r="O278" s="100"/>
+    <row r="275" s="6" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J275" s="100"/>
+      <c r="L275" s="100"/>
+      <c r="M275" s="100"/>
+      <c r="O275" s="100"/>
+    </row>
+    <row r="276" s="6" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J276" s="100"/>
+      <c r="L276" s="100"/>
+      <c r="M276" s="100"/>
+      <c r="O276" s="100"/>
+    </row>
+    <row r="277" s="11" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J277" s="106"/>
+      <c r="L277" s="106"/>
+      <c r="M277" s="106"/>
+      <c r="O277" s="106"/>
+    </row>
+    <row r="278" s="12" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J278" s="107"/>
+      <c r="L278" s="107"/>
+      <c r="M278" s="107"/>
+      <c r="O278" s="107"/>
     </row>
     <row r="279" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J279" s="100"/>
@@ -7943,115 +8016,107 @@
       <c r="M304" s="100"/>
       <c r="O304" s="100"/>
     </row>
-    <row r="305" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="305" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J305" s="100"/>
       <c r="L305" s="100"/>
       <c r="M305" s="100"/>
       <c r="O305" s="100"/>
     </row>
-    <row r="306" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="306" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J306" s="100"/>
       <c r="L306" s="100"/>
       <c r="M306" s="100"/>
       <c r="O306" s="100"/>
     </row>
-    <row r="307" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="307" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J307" s="100"/>
       <c r="L307" s="100"/>
       <c r="M307" s="100"/>
       <c r="O307" s="100"/>
     </row>
-    <row r="308" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="308" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J308" s="100"/>
       <c r="L308" s="100"/>
       <c r="M308" s="100"/>
       <c r="O308" s="100"/>
     </row>
-    <row r="309" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="309" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J309" s="100"/>
       <c r="L309" s="100"/>
       <c r="M309" s="100"/>
       <c r="O309" s="100"/>
     </row>
-    <row r="310" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="310" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J310" s="100"/>
       <c r="L310" s="100"/>
       <c r="M310" s="100"/>
       <c r="O310" s="100"/>
     </row>
-    <row r="311" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="311" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J311" s="100"/>
       <c r="L311" s="100"/>
       <c r="M311" s="100"/>
       <c r="O311" s="100"/>
     </row>
-    <row r="312" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="312" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J312" s="100"/>
       <c r="L312" s="100"/>
       <c r="M312" s="100"/>
       <c r="O312" s="100"/>
     </row>
-    <row r="313" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="313" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J313" s="100"/>
       <c r="L313" s="100"/>
       <c r="M313" s="100"/>
       <c r="O313" s="100"/>
     </row>
-    <row r="314" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="314" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J314" s="100"/>
       <c r="L314" s="100"/>
       <c r="M314" s="100"/>
       <c r="O314" s="100"/>
     </row>
-    <row r="315" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="315" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J315" s="100"/>
       <c r="L315" s="100"/>
       <c r="M315" s="100"/>
       <c r="O315" s="100"/>
     </row>
-    <row r="316" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="316" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J316" s="100"/>
       <c r="L316" s="100"/>
       <c r="M316" s="100"/>
       <c r="O316" s="100"/>
     </row>
-    <row r="317" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="317" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J317" s="100"/>
       <c r="L317" s="100"/>
       <c r="M317" s="100"/>
       <c r="O317" s="100"/>
     </row>
-    <row r="318" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="318" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J318" s="100"/>
       <c r="L318" s="100"/>
       <c r="M318" s="100"/>
       <c r="O318" s="100"/>
     </row>
-    <row r="319" s="6" customFormat="1" customHeight="1" spans="9:29">
+    <row r="319" s="6" customFormat="1" customHeight="1" spans="10:15">
       <c r="J319" s="100"/>
       <c r="L319" s="100"/>
       <c r="M319" s="100"/>
       <c r="O319" s="100"/>
     </row>
-    <row r="320" s="6" customFormat="1" customHeight="1" spans="9:29">
-      <c r="I320" s="19"/>
-      <c r="J320" s="108"/>
-      <c r="K320" s="19"/>
-      <c r="L320" s="108"/>
+    <row r="320" s="6" customFormat="1" customHeight="1" spans="10:15">
+      <c r="J320" s="100"/>
+      <c r="L320" s="100"/>
       <c r="M320" s="100"/>
-      <c r="N320" s="19"/>
-      <c r="O320" s="108"/>
-      <c r="AC320" s="100"/>
+      <c r="O320" s="100"/>
     </row>
     <row r="321" s="6" customFormat="1" customHeight="1" spans="9:29">
-      <c r="I321" s="19"/>
-      <c r="J321" s="108"/>
-      <c r="K321" s="19"/>
-      <c r="L321" s="108"/>
+      <c r="J321" s="100"/>
+      <c r="L321" s="100"/>
       <c r="M321" s="100"/>
-      <c r="N321" s="19"/>
-      <c r="O321" s="108"/>
-      <c r="AC321" s="100"/>
+      <c r="O321" s="100"/>
     </row>
     <row r="322" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I322" s="19"/>
@@ -9803,7 +9868,7 @@
       <c r="O496" s="108"/>
       <c r="AC496" s="100"/>
     </row>
-    <row r="497" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="497" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I497" s="19"/>
       <c r="J497" s="108"/>
       <c r="K497" s="19"/>
@@ -9813,7 +9878,7 @@
       <c r="O497" s="108"/>
       <c r="AC497" s="100"/>
     </row>
-    <row r="498" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="498" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I498" s="19"/>
       <c r="J498" s="108"/>
       <c r="K498" s="19"/>
@@ -9823,7 +9888,7 @@
       <c r="O498" s="108"/>
       <c r="AC498" s="100"/>
     </row>
-    <row r="499" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="499" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I499" s="19"/>
       <c r="J499" s="108"/>
       <c r="K499" s="19"/>
@@ -9833,7 +9898,7 @@
       <c r="O499" s="108"/>
       <c r="AC499" s="100"/>
     </row>
-    <row r="500" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="500" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I500" s="19"/>
       <c r="J500" s="108"/>
       <c r="K500" s="19"/>
@@ -9843,7 +9908,7 @@
       <c r="O500" s="108"/>
       <c r="AC500" s="100"/>
     </row>
-    <row r="501" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="501" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I501" s="19"/>
       <c r="J501" s="108"/>
       <c r="K501" s="19"/>
@@ -9853,7 +9918,7 @@
       <c r="O501" s="108"/>
       <c r="AC501" s="100"/>
     </row>
-    <row r="502" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="502" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I502" s="19"/>
       <c r="J502" s="108"/>
       <c r="K502" s="19"/>
@@ -9863,7 +9928,7 @@
       <c r="O502" s="108"/>
       <c r="AC502" s="100"/>
     </row>
-    <row r="503" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="503" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I503" s="19"/>
       <c r="J503" s="108"/>
       <c r="K503" s="19"/>
@@ -9873,7 +9938,7 @@
       <c r="O503" s="108"/>
       <c r="AC503" s="100"/>
     </row>
-    <row r="504" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="504" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I504" s="19"/>
       <c r="J504" s="108"/>
       <c r="K504" s="19"/>
@@ -9883,7 +9948,7 @@
       <c r="O504" s="108"/>
       <c r="AC504" s="100"/>
     </row>
-    <row r="505" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="505" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I505" s="19"/>
       <c r="J505" s="108"/>
       <c r="K505" s="19"/>
@@ -9893,7 +9958,7 @@
       <c r="O505" s="108"/>
       <c r="AC505" s="100"/>
     </row>
-    <row r="506" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="506" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I506" s="19"/>
       <c r="J506" s="108"/>
       <c r="K506" s="19"/>
@@ -9903,7 +9968,7 @@
       <c r="O506" s="108"/>
       <c r="AC506" s="100"/>
     </row>
-    <row r="507" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="507" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I507" s="19"/>
       <c r="J507" s="108"/>
       <c r="K507" s="19"/>
@@ -9913,7 +9978,7 @@
       <c r="O507" s="108"/>
       <c r="AC507" s="100"/>
     </row>
-    <row r="508" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="508" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I508" s="19"/>
       <c r="J508" s="108"/>
       <c r="K508" s="19"/>
@@ -9923,7 +9988,7 @@
       <c r="O508" s="108"/>
       <c r="AC508" s="100"/>
     </row>
-    <row r="509" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="509" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I509" s="19"/>
       <c r="J509" s="108"/>
       <c r="K509" s="19"/>
@@ -9933,7 +9998,7 @@
       <c r="O509" s="108"/>
       <c r="AC509" s="100"/>
     </row>
-    <row r="510" s="6" customFormat="1" customHeight="1" spans="1:32">
+    <row r="510" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I510" s="19"/>
       <c r="J510" s="108"/>
       <c r="K510" s="19"/>
@@ -9943,15 +10008,7 @@
       <c r="O510" s="108"/>
       <c r="AC510" s="100"/>
     </row>
-    <row r="511" customHeight="1" spans="1:32">
-      <c r="A511" s="6"/>
-      <c r="B511" s="6"/>
-      <c r="C511" s="6"/>
-      <c r="D511" s="6"/>
-      <c r="E511" s="6"/>
-      <c r="F511" s="6"/>
-      <c r="G511" s="6"/>
-      <c r="H511" s="6"/>
+    <row r="511" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I511" s="19"/>
       <c r="J511" s="108"/>
       <c r="K511" s="19"/>
@@ -9959,33 +10016,9 @@
       <c r="M511" s="100"/>
       <c r="N511" s="19"/>
       <c r="O511" s="108"/>
-      <c r="P511" s="6"/>
-      <c r="Q511" s="6"/>
-      <c r="R511" s="6"/>
-      <c r="S511" s="6"/>
-      <c r="T511" s="6"/>
-      <c r="U511" s="6"/>
-      <c r="V511" s="6"/>
-      <c r="W511" s="6"/>
-      <c r="X511" s="6"/>
-      <c r="Y511" s="6"/>
-      <c r="Z511" s="6"/>
-      <c r="AA511" s="6"/>
-      <c r="AB511" s="6"/>
       <c r="AC511" s="100"/>
-      <c r="AD511" s="6"/>
-      <c r="AE511" s="6"/>
-      <c r="AF511" s="6"/>
-    </row>
-    <row r="512" customHeight="1" spans="1:32">
-      <c r="A512" s="6"/>
-      <c r="B512" s="6"/>
-      <c r="C512" s="6"/>
-      <c r="D512" s="6"/>
-      <c r="E512" s="6"/>
-      <c r="F512" s="6"/>
-      <c r="G512" s="6"/>
-      <c r="H512" s="6"/>
+    </row>
+    <row r="512" s="6" customFormat="1" customHeight="1" spans="9:29">
       <c r="I512" s="19"/>
       <c r="J512" s="108"/>
       <c r="K512" s="19"/>
@@ -9993,23 +10026,7 @@
       <c r="M512" s="100"/>
       <c r="N512" s="19"/>
       <c r="O512" s="108"/>
-      <c r="P512" s="6"/>
-      <c r="Q512" s="6"/>
-      <c r="R512" s="6"/>
-      <c r="S512" s="6"/>
-      <c r="T512" s="6"/>
-      <c r="U512" s="6"/>
-      <c r="V512" s="6"/>
-      <c r="W512" s="6"/>
-      <c r="X512" s="6"/>
-      <c r="Y512" s="6"/>
-      <c r="Z512" s="6"/>
-      <c r="AA512" s="6"/>
-      <c r="AB512" s="6"/>
       <c r="AC512" s="100"/>
-      <c r="AD512" s="6"/>
-      <c r="AE512" s="6"/>
-      <c r="AF512" s="6"/>
     </row>
     <row r="513" customHeight="1" spans="1:32">
       <c r="A513" s="6"/>
@@ -10214,6 +10231,74 @@
       <c r="AD518" s="6"/>
       <c r="AE518" s="6"/>
       <c r="AF518" s="6"/>
+    </row>
+    <row r="519" customHeight="1" spans="1:32">
+      <c r="A519" s="6"/>
+      <c r="B519" s="6"/>
+      <c r="C519" s="6"/>
+      <c r="D519" s="6"/>
+      <c r="E519" s="6"/>
+      <c r="F519" s="6"/>
+      <c r="G519" s="6"/>
+      <c r="H519" s="6"/>
+      <c r="I519" s="19"/>
+      <c r="J519" s="108"/>
+      <c r="K519" s="19"/>
+      <c r="L519" s="108"/>
+      <c r="M519" s="100"/>
+      <c r="N519" s="19"/>
+      <c r="O519" s="108"/>
+      <c r="P519" s="6"/>
+      <c r="Q519" s="6"/>
+      <c r="R519" s="6"/>
+      <c r="S519" s="6"/>
+      <c r="T519" s="6"/>
+      <c r="U519" s="6"/>
+      <c r="V519" s="6"/>
+      <c r="W519" s="6"/>
+      <c r="X519" s="6"/>
+      <c r="Y519" s="6"/>
+      <c r="Z519" s="6"/>
+      <c r="AA519" s="6"/>
+      <c r="AB519" s="6"/>
+      <c r="AC519" s="100"/>
+      <c r="AD519" s="6"/>
+      <c r="AE519" s="6"/>
+      <c r="AF519" s="6"/>
+    </row>
+    <row r="520" customHeight="1" spans="1:32">
+      <c r="A520" s="6"/>
+      <c r="B520" s="6"/>
+      <c r="C520" s="6"/>
+      <c r="D520" s="6"/>
+      <c r="E520" s="6"/>
+      <c r="F520" s="6"/>
+      <c r="G520" s="6"/>
+      <c r="H520" s="6"/>
+      <c r="I520" s="19"/>
+      <c r="J520" s="108"/>
+      <c r="K520" s="19"/>
+      <c r="L520" s="108"/>
+      <c r="M520" s="100"/>
+      <c r="N520" s="19"/>
+      <c r="O520" s="108"/>
+      <c r="P520" s="6"/>
+      <c r="Q520" s="6"/>
+      <c r="R520" s="6"/>
+      <c r="S520" s="6"/>
+      <c r="T520" s="6"/>
+      <c r="U520" s="6"/>
+      <c r="V520" s="6"/>
+      <c r="W520" s="6"/>
+      <c r="X520" s="6"/>
+      <c r="Y520" s="6"/>
+      <c r="Z520" s="6"/>
+      <c r="AA520" s="6"/>
+      <c r="AB520" s="6"/>
+      <c r="AC520" s="100"/>
+      <c r="AD520" s="6"/>
+      <c r="AE520" s="6"/>
+      <c r="AF520" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="39">

</xml_diff>